<commit_message>
Month-end for every month, deliberate period locks, Calls downloads from templates
- Period-lock register (Data/Common/period_lock.csv, tools/lock_period.py): a month is Locked only when
  someone locks it; reports and the home dashboard default to the most recent locked month. Statuses show
  the reported month only.
- month_end.py: balance sheet and cash flow for every month end, Oct 2024 to Sep 2026, joining the locked
  model at 31 Jul 2026 to the dollar (fact_balance_month, fact_cash_flow_month). Home dashboard shows all
  three statements for every month. History fixes: services milestone billing, finished grants' instalments,
  no duplicate May-Jul services invoices. P&L unchanged.
- Calls report: Excel, PDF and PowerPoint made on click from templates (assets/exports/), no pre-built files.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/media/exports/nfp-sample-statements.xlsx
+++ b/media/exports/nfp-sample-statements.xlsx
@@ -948,7 +948,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Data status: Sep 2026 locked · Aug 2026 locked · Oct 2026 incomplete (data retrieved 2pm, Tue 6 Oct 2026) · Generated 9 Oct 2026, 8:56am</t>
+          <t>Data status: Sep 2026 locked (data retrieved 2pm, Tue 6 Oct 2026) · Generated 22 Oct 2026, 4:57pm</t>
         </is>
       </c>
     </row>
@@ -1165,7 +1165,7 @@
   <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
     <oddHeader>&amp;L&amp;"Roboto,Regular"&amp;8 Sample Community Services Ltd&amp;R&amp;"Roboto,Regular"&amp;8 &amp;A</oddHeader>
-    <oddFooter>&amp;L&amp;"Roboto,Regular"&amp;8 nfp-sample-statements.xlsx&amp;C&amp;"Roboto,Regular"&amp;8 Data retrieved 2pm, Tue 6 Oct 2026 · Generated 9 Oct 2026, 8:56am&amp;R&amp;"Roboto,Regular"&amp;8 Page &amp;P of &amp;N</oddFooter>
+    <oddFooter>&amp;L&amp;"Roboto,Regular"&amp;8 nfp-sample-statements.xlsx&amp;C&amp;"Roboto,Regular"&amp;8 Data retrieved 2pm, Tue 6 Oct 2026 · Generated 22 Oct 2026, 4:57pm&amp;R&amp;"Roboto,Regular"&amp;8 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -1207,7 +1207,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Data status: Sep 2026 locked · Aug 2026 locked · Oct 2026 incomplete (data retrieved 2pm, Tue 6 Oct 2026) · Generated 9 Oct 2026, 8:56am</t>
+          <t>Data status: Sep 2026 locked (data retrieved 2pm, Tue 6 Oct 2026) · Generated 22 Oct 2026, 4:57pm</t>
         </is>
       </c>
     </row>
@@ -1954,7 +1954,7 @@
   <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
     <oddHeader>&amp;L&amp;"Roboto,Regular"&amp;8 Sample Community Services Ltd&amp;R&amp;"Roboto,Regular"&amp;8 &amp;A</oddHeader>
-    <oddFooter>&amp;L&amp;"Roboto,Regular"&amp;8 nfp-sample-statements.xlsx&amp;C&amp;"Roboto,Regular"&amp;8 Data retrieved 2pm, Tue 6 Oct 2026 · Generated 9 Oct 2026, 8:56am&amp;R&amp;"Roboto,Regular"&amp;8 Page &amp;P of &amp;N</oddFooter>
+    <oddFooter>&amp;L&amp;"Roboto,Regular"&amp;8 nfp-sample-statements.xlsx&amp;C&amp;"Roboto,Regular"&amp;8 Data retrieved 2pm, Tue 6 Oct 2026 · Generated 22 Oct 2026, 4:57pm&amp;R&amp;"Roboto,Regular"&amp;8 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -1998,7 +1998,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Data status: Sep 2026 locked · Aug 2026 locked · Oct 2026 incomplete (data retrieved 2pm, Tue 6 Oct 2026) · Generated 9 Oct 2026, 8:56am</t>
+          <t>Data status: Sep 2026 locked (data retrieved 2pm, Tue 6 Oct 2026) · Generated 22 Oct 2026, 4:57pm</t>
         </is>
       </c>
     </row>
@@ -2348,7 +2348,7 @@
   <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
     <oddHeader>&amp;L&amp;"Roboto,Regular"&amp;8 Sample Community Services Ltd&amp;R&amp;"Roboto,Regular"&amp;8 &amp;A</oddHeader>
-    <oddFooter>&amp;L&amp;"Roboto,Regular"&amp;8 nfp-sample-statements.xlsx&amp;C&amp;"Roboto,Regular"&amp;8 Data retrieved 2pm, Tue 6 Oct 2026 · Generated 9 Oct 2026, 8:56am&amp;R&amp;"Roboto,Regular"&amp;8 Page &amp;P of &amp;N</oddFooter>
+    <oddFooter>&amp;L&amp;"Roboto,Regular"&amp;8 nfp-sample-statements.xlsx&amp;C&amp;"Roboto,Regular"&amp;8 Data retrieved 2pm, Tue 6 Oct 2026 · Generated 22 Oct 2026, 4:57pm&amp;R&amp;"Roboto,Regular"&amp;8 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -2389,7 +2389,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Data status: Sep 2026 locked · Aug 2026 locked · Oct 2026 incomplete (data retrieved 2pm, Tue 6 Oct 2026) · Generated 9 Oct 2026, 8:56am</t>
+          <t>Data status: Sep 2026 locked (data retrieved 2pm, Tue 6 Oct 2026) · Generated 22 Oct 2026, 4:57pm</t>
         </is>
       </c>
     </row>
@@ -2768,7 +2768,7 @@
   <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
     <oddHeader>&amp;L&amp;"Roboto,Regular"&amp;8 Sample Community Services Ltd&amp;R&amp;"Roboto,Regular"&amp;8 &amp;A</oddHeader>
-    <oddFooter>&amp;L&amp;"Roboto,Regular"&amp;8 nfp-sample-statements.xlsx&amp;C&amp;"Roboto,Regular"&amp;8 Data retrieved 2pm, Tue 6 Oct 2026 · Generated 9 Oct 2026, 8:56am&amp;R&amp;"Roboto,Regular"&amp;8 Page &amp;P of &amp;N</oddFooter>
+    <oddFooter>&amp;L&amp;"Roboto,Regular"&amp;8 nfp-sample-statements.xlsx&amp;C&amp;"Roboto,Regular"&amp;8 Data retrieved 2pm, Tue 6 Oct 2026 · Generated 22 Oct 2026, 4:57pm&amp;R&amp;"Roboto,Regular"&amp;8 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -2818,7 +2818,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Data status: Sep 2026 locked · Aug 2026 locked · Oct 2026 incomplete (data retrieved 2pm, Tue 6 Oct 2026) · Generated 9 Oct 2026, 8:56am</t>
+          <t>Data status: Sep 2026 locked (data retrieved 2pm, Tue 6 Oct 2026) · Generated 22 Oct 2026, 4:57pm</t>
         </is>
       </c>
     </row>
@@ -3220,7 +3220,7 @@
   <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
     <oddHeader>&amp;L&amp;"Roboto,Regular"&amp;8 Sample Community Services Ltd&amp;R&amp;"Roboto,Regular"&amp;8 &amp;A</oddHeader>
-    <oddFooter>&amp;L&amp;"Roboto,Regular"&amp;8 nfp-sample-statements.xlsx&amp;C&amp;"Roboto,Regular"&amp;8 Data retrieved 2pm, Tue 6 Oct 2026 · Generated 9 Oct 2026, 8:56am&amp;R&amp;"Roboto,Regular"&amp;8 Page &amp;P of &amp;N</oddFooter>
+    <oddFooter>&amp;L&amp;"Roboto,Regular"&amp;8 nfp-sample-statements.xlsx&amp;C&amp;"Roboto,Regular"&amp;8 Data retrieved 2pm, Tue 6 Oct 2026 · Generated 22 Oct 2026, 4:57pm&amp;R&amp;"Roboto,Regular"&amp;8 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -3265,7 +3265,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Data status: Sep 2026 locked · Aug 2026 locked · Oct 2026 incomplete (data retrieved 2pm, Tue 6 Oct 2026) · Generated 9 Oct 2026, 8:56am</t>
+          <t>Data status: Sep 2026 locked (data retrieved 2pm, Tue 6 Oct 2026) · Generated 22 Oct 2026, 4:57pm</t>
         </is>
       </c>
     </row>
@@ -5456,7 +5456,7 @@
   <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
     <oddHeader>&amp;L&amp;"Roboto,Regular"&amp;8 Sample Community Services Ltd&amp;R&amp;"Roboto,Regular"&amp;8 &amp;A</oddHeader>
-    <oddFooter>&amp;L&amp;"Roboto,Regular"&amp;8 nfp-sample-statements.xlsx&amp;C&amp;"Roboto,Regular"&amp;8 Data retrieved 2pm, Tue 6 Oct 2026 · Generated 9 Oct 2026, 8:56am&amp;R&amp;"Roboto,Regular"&amp;8 Page &amp;P of &amp;N</oddFooter>
+    <oddFooter>&amp;L&amp;"Roboto,Regular"&amp;8 nfp-sample-statements.xlsx&amp;C&amp;"Roboto,Regular"&amp;8 Data retrieved 2pm, Tue 6 Oct 2026 · Generated 22 Oct 2026, 4:57pm&amp;R&amp;"Roboto,Regular"&amp;8 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -5504,7 +5504,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Data status: Sep 2026 locked · Aug 2026 locked · Oct 2026 incomplete (data retrieved 2pm, Tue 6 Oct 2026) · Generated 9 Oct 2026, 8:56am</t>
+          <t>Data status: Sep 2026 locked (data retrieved 2pm, Tue 6 Oct 2026) · Generated 22 Oct 2026, 4:57pm</t>
         </is>
       </c>
     </row>
@@ -6009,7 +6009,7 @@
   <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
     <oddHeader>&amp;L&amp;"Roboto,Regular"&amp;8 Sample Community Services Ltd&amp;R&amp;"Roboto,Regular"&amp;8 &amp;A</oddHeader>
-    <oddFooter>&amp;L&amp;"Roboto,Regular"&amp;8 nfp-sample-statements.xlsx&amp;C&amp;"Roboto,Regular"&amp;8 Data retrieved 2pm, Tue 6 Oct 2026 · Generated 9 Oct 2026, 8:56am&amp;R&amp;"Roboto,Regular"&amp;8 Page &amp;P of &amp;N</oddFooter>
+    <oddFooter>&amp;L&amp;"Roboto,Regular"&amp;8 nfp-sample-statements.xlsx&amp;C&amp;"Roboto,Regular"&amp;8 Data retrieved 2pm, Tue 6 Oct 2026 · Generated 22 Oct 2026, 4:57pm&amp;R&amp;"Roboto,Regular"&amp;8 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>

</xml_diff>